<commit_message>
chore: sync brand deck v4.6, pricing artifacts, and probation deck
Tighten the Trinity brand sales deck to 18 pages (scene+path merge, combo visuals, CTA into billing), refresh pricing docs/outputs/scripts, and add probation答辩 materials and weekly notes.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/pricing/output/trinity-pricing-image.xlsx
+++ b/pricing/output/trinity-pricing-image.xlsx
@@ -560,10 +560,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -595,10 +595,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -844,7 +844,7 @@
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
     <col min="5" max="5" width="10.83203125" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="11.83203125" customWidth="1"/>
     <col min="8" max="8" width="24.83203125" customWidth="1"/>
     <col min="9" max="9" width="10.83203125" customWidth="1"/>
     <col min="10" max="10" width="12.83203125" customWidth="1"/>
@@ -1672,10 +1672,10 @@
         <v>$0.211/张</v>
       </c>
       <c r="G16" s="10" t="str">
-        <v>¥1.583/张</v>
+        <v>—</v>
       </c>
       <c r="H16" s="10" t="str">
-        <v>$0.211/张</v>
+        <v>—</v>
       </c>
       <c r="I16" s="10" t="str">
         <v>—</v>
@@ -1684,13 +1684,13 @@
         <v>—</v>
       </c>
       <c r="K16" s="10" t="str">
-        <v>$0.211/张</v>
+        <v>—</v>
       </c>
       <c r="L16" s="10" t="str">
         <v>—</v>
       </c>
       <c r="M16" s="10" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="N16" s="10" t="str">
         <v>—</v>
@@ -1699,7 +1699,7 @@
         <v>—</v>
       </c>
       <c r="P16" s="10" t="str">
-        <v>价✅</v>
+        <v>— 未上架</v>
       </c>
       <c r="Q16" s="10" t="str">
         <v/>
@@ -1725,10 +1725,10 @@
         <v>$0.428/张</v>
       </c>
       <c r="G17" s="9" t="str">
-        <v>¥3.21/张</v>
+        <v>—</v>
       </c>
       <c r="H17" s="9" t="str">
-        <v>$0.428/张</v>
+        <v>—</v>
       </c>
       <c r="I17" s="9" t="str">
         <v>—</v>
@@ -1737,13 +1737,13 @@
         <v>—</v>
       </c>
       <c r="K17" s="9" t="str">
-        <v>$0.428/张</v>
+        <v>—</v>
       </c>
       <c r="L17" s="9" t="str">
         <v>—</v>
       </c>
       <c r="M17" s="9" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="N17" s="9" t="str">
         <v>—</v>
@@ -1752,7 +1752,7 @@
         <v>—</v>
       </c>
       <c r="P17" s="9" t="str">
-        <v>价✅</v>
+        <v>— 未上架</v>
       </c>
       <c r="Q17" s="9" t="str">
         <v/>
@@ -1778,10 +1778,10 @@
         <v>$0.712/张</v>
       </c>
       <c r="G18" s="9" t="str">
-        <v>¥5.34/张</v>
+        <v>—</v>
       </c>
       <c r="H18" s="9" t="str">
-        <v>$0.712/张</v>
+        <v>—</v>
       </c>
       <c r="I18" s="9" t="str">
         <v>—</v>
@@ -1790,13 +1790,13 @@
         <v>—</v>
       </c>
       <c r="K18" s="9" t="str">
-        <v>$0.712/张</v>
+        <v>—</v>
       </c>
       <c r="L18" s="9" t="str">
         <v>—</v>
       </c>
       <c r="M18" s="9" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="N18" s="9" t="str">
         <v>—</v>
@@ -1805,7 +1805,7 @@
         <v>—</v>
       </c>
       <c r="P18" s="9" t="str">
-        <v>价✅</v>
+        <v>— 未上架</v>
       </c>
       <c r="Q18" s="9" t="str">
         <v/>
@@ -1831,10 +1831,10 @@
         <v>$0.006/张</v>
       </c>
       <c r="G19" s="9" t="str">
-        <v>¥0.045/张</v>
+        <v>—</v>
       </c>
       <c r="H19" s="9" t="str">
-        <v>$0.006/张</v>
+        <v>—</v>
       </c>
       <c r="I19" s="9" t="str">
         <v>—</v>
@@ -1843,13 +1843,13 @@
         <v>—</v>
       </c>
       <c r="K19" s="9" t="str">
-        <v>$0.006/张</v>
+        <v>—</v>
       </c>
       <c r="L19" s="9" t="str">
         <v>—</v>
       </c>
       <c r="M19" s="9" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="N19" s="9" t="str">
         <v>—</v>
@@ -1858,7 +1858,7 @@
         <v>—</v>
       </c>
       <c r="P19" s="9" t="str">
-        <v>价✅</v>
+        <v>— 未上架</v>
       </c>
       <c r="Q19" s="9" t="str">
         <v/>
@@ -1884,10 +1884,10 @@
         <v>$0.012/张</v>
       </c>
       <c r="G20" s="9" t="str">
-        <v>¥0.09/张</v>
+        <v>—</v>
       </c>
       <c r="H20" s="9" t="str">
-        <v>$0.012/张</v>
+        <v>—</v>
       </c>
       <c r="I20" s="9" t="str">
         <v>—</v>
@@ -1896,13 +1896,13 @@
         <v>—</v>
       </c>
       <c r="K20" s="9" t="str">
-        <v>$0.012/张</v>
+        <v>—</v>
       </c>
       <c r="L20" s="9" t="str">
         <v>—</v>
       </c>
       <c r="M20" s="9" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="N20" s="9" t="str">
         <v>—</v>
@@ -1911,7 +1911,7 @@
         <v>—</v>
       </c>
       <c r="P20" s="9" t="str">
-        <v>价✅</v>
+        <v>— 未上架</v>
       </c>
       <c r="Q20" s="9" t="str">
         <v/>
@@ -1937,10 +1937,10 @@
         <v>$0.02/张</v>
       </c>
       <c r="G21" s="9" t="str">
-        <v>¥0.15/张</v>
+        <v>—</v>
       </c>
       <c r="H21" s="9" t="str">
-        <v>$0.02/张</v>
+        <v>—</v>
       </c>
       <c r="I21" s="9" t="str">
         <v>—</v>
@@ -1949,13 +1949,13 @@
         <v>—</v>
       </c>
       <c r="K21" s="9" t="str">
-        <v>$0.02/张</v>
+        <v>—</v>
       </c>
       <c r="L21" s="9" t="str">
         <v>—</v>
       </c>
       <c r="M21" s="9" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="N21" s="9" t="str">
         <v>—</v>
@@ -1964,7 +1964,7 @@
         <v>—</v>
       </c>
       <c r="P21" s="9" t="str">
-        <v>价✅</v>
+        <v>— 未上架</v>
       </c>
       <c r="Q21" s="9" t="str">
         <v/>
@@ -1990,10 +1990,10 @@
         <v>$0.053/张</v>
       </c>
       <c r="G22" s="9" t="str">
-        <v>¥0.398/张</v>
+        <v>—</v>
       </c>
       <c r="H22" s="9" t="str">
-        <v>$0.053/张</v>
+        <v>—</v>
       </c>
       <c r="I22" s="9" t="str">
         <v>—</v>
@@ -2002,13 +2002,13 @@
         <v>—</v>
       </c>
       <c r="K22" s="9" t="str">
-        <v>$0.053/张</v>
+        <v>—</v>
       </c>
       <c r="L22" s="9" t="str">
         <v>—</v>
       </c>
       <c r="M22" s="9" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="N22" s="9" t="str">
         <v>—</v>
@@ -2017,7 +2017,7 @@
         <v>—</v>
       </c>
       <c r="P22" s="9" t="str">
-        <v>价✅</v>
+        <v>— 未上架</v>
       </c>
       <c r="Q22" s="9" t="str">
         <v/>
@@ -2043,10 +2043,10 @@
         <v>$0.107/张</v>
       </c>
       <c r="G23" s="9" t="str">
-        <v>¥0.803/张</v>
+        <v>—</v>
       </c>
       <c r="H23" s="9" t="str">
-        <v>$0.107/张</v>
+        <v>—</v>
       </c>
       <c r="I23" s="9" t="str">
         <v>—</v>
@@ -2055,13 +2055,13 @@
         <v>—</v>
       </c>
       <c r="K23" s="9" t="str">
-        <v>$0.107/张</v>
+        <v>—</v>
       </c>
       <c r="L23" s="9" t="str">
         <v>—</v>
       </c>
       <c r="M23" s="9" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="N23" s="9" t="str">
         <v>—</v>
@@ -2070,7 +2070,7 @@
         <v>—</v>
       </c>
       <c r="P23" s="9" t="str">
-        <v>价✅</v>
+        <v>— 未上架</v>
       </c>
       <c r="Q23" s="9" t="str">
         <v/>
@@ -2096,10 +2096,10 @@
         <v>$0.178/张</v>
       </c>
       <c r="G24" s="9" t="str">
-        <v>¥1.335/张</v>
+        <v>—</v>
       </c>
       <c r="H24" s="9" t="str">
-        <v>$0.178/张</v>
+        <v>—</v>
       </c>
       <c r="I24" s="9" t="str">
         <v>—</v>
@@ -2108,13 +2108,13 @@
         <v>—</v>
       </c>
       <c r="K24" s="9" t="str">
-        <v>$0.178/张</v>
+        <v>—</v>
       </c>
       <c r="L24" s="9" t="str">
         <v>—</v>
       </c>
       <c r="M24" s="9" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="N24" s="9" t="str">
         <v>—</v>
@@ -2123,7 +2123,7 @@
         <v>—</v>
       </c>
       <c r="P24" s="9" t="str">
-        <v>价✅</v>
+        <v>— 未上架</v>
       </c>
       <c r="Q24" s="9" t="str">
         <v/>
@@ -2149,10 +2149,10 @@
         <v>¥0.1875/张</v>
       </c>
       <c r="G25" s="12" t="str">
-        <v>¥0.1875/张</v>
+        <v>—</v>
       </c>
       <c r="H25" s="12" t="str">
-        <v>$0.0288461538461539/张</v>
+        <v>—</v>
       </c>
       <c r="I25" s="12" t="str">
         <v>—</v>
@@ -2161,13 +2161,13 @@
         <v>—</v>
       </c>
       <c r="K25" s="12" t="str">
-        <v>$0.0289/张</v>
+        <v>—</v>
       </c>
       <c r="L25" s="12" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="M25" s="12" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="N25" s="12" t="str">
         <v>—</v>
@@ -2176,7 +2176,7 @@
         <v>—</v>
       </c>
       <c r="P25" s="12" t="str">
-        <v>价✅</v>
+        <v>— 未上架</v>
       </c>
       <c r="Q25" s="12" t="str">
         <v>viduq2 文生图 · 积分计价</v>
@@ -2202,10 +2202,10 @@
         <v>¥0.25/张</v>
       </c>
       <c r="G26" s="11" t="str">
-        <v>¥0.25/张</v>
+        <v>—</v>
       </c>
       <c r="H26" s="11" t="str">
-        <v>$0.0384615384615385/张</v>
+        <v>—</v>
       </c>
       <c r="I26" s="11" t="str">
         <v>—</v>
@@ -2214,13 +2214,13 @@
         <v>—</v>
       </c>
       <c r="K26" s="11" t="str">
-        <v>$0.0385/张</v>
+        <v>—</v>
       </c>
       <c r="L26" s="11" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="M26" s="11" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="N26" s="11" t="str">
         <v>—</v>
@@ -2229,7 +2229,7 @@
         <v>—</v>
       </c>
       <c r="P26" s="11" t="str">
-        <v>价✅</v>
+        <v>— 未上架</v>
       </c>
       <c r="Q26" s="11" t="str">
         <v>viduq2 文生图 · 积分计价</v>
@@ -2255,10 +2255,10 @@
         <v>¥0.3125/张</v>
       </c>
       <c r="G27" s="11" t="str">
-        <v>¥0.3125/张</v>
+        <v>—</v>
       </c>
       <c r="H27" s="11" t="str">
-        <v>$0.0480769230769231/张</v>
+        <v>—</v>
       </c>
       <c r="I27" s="11" t="str">
         <v>—</v>
@@ -2267,13 +2267,13 @@
         <v>—</v>
       </c>
       <c r="K27" s="11" t="str">
-        <v>$0.0481/张</v>
+        <v>—</v>
       </c>
       <c r="L27" s="11" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="M27" s="11" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="N27" s="11" t="str">
         <v>—</v>
@@ -2282,7 +2282,7 @@
         <v>—</v>
       </c>
       <c r="P27" s="11" t="str">
-        <v>价✅</v>
+        <v>— 未上架</v>
       </c>
       <c r="Q27" s="11" t="str">
         <v>viduq2 文生图 · 积分计价</v>
@@ -4960,7 +4960,7 @@
     </row>
     <row r="23">
       <c r="A23" s="21" t="str">
-        <v>生成时间：2026-08-07T10:56:45Z</v>
+        <v>生成时间：2026-08-18T07:48:14Z</v>
       </c>
       <c r="B23" s="21" t="str">
         <v/>
@@ -6288,13 +6288,13 @@
         <v>¥0.1/张</v>
       </c>
       <c r="G43" s="17" t="str">
-        <v>$0.006</v>
+        <v>—</v>
       </c>
       <c r="H43" s="17" t="str">
         <v>—</v>
       </c>
       <c r="I43" s="17" t="str">
-        <v>⚠+156.4%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="44">
@@ -6317,13 +6317,13 @@
         <v>¥0.045/张</v>
       </c>
       <c r="G44" s="17" t="str">
-        <v>$0.006</v>
+        <v>—</v>
       </c>
       <c r="H44" s="17" t="str">
         <v>—</v>
       </c>
       <c r="I44" s="17" t="str">
-        <v>⚠+15.4%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="45">
@@ -6346,13 +6346,13 @@
         <v>¥0.09/张</v>
       </c>
       <c r="G45" s="17" t="str">
-        <v>$0.012</v>
+        <v>—</v>
       </c>
       <c r="H45" s="17" t="str">
         <v>—</v>
       </c>
       <c r="I45" s="17" t="str">
-        <v>⚠+15.4%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="46">
@@ -6375,13 +6375,13 @@
         <v>¥0.15/张</v>
       </c>
       <c r="G46" s="17" t="str">
-        <v>$0.02</v>
+        <v>—</v>
       </c>
       <c r="H46" s="17" t="str">
         <v>—</v>
       </c>
       <c r="I46" s="17" t="str">
-        <v>⚠+15.4%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="47">
@@ -6404,13 +6404,13 @@
         <v>¥0.398/张</v>
       </c>
       <c r="G47" s="17" t="str">
-        <v>$0.006</v>
+        <v>—</v>
       </c>
       <c r="H47" s="17" t="str">
         <v>—</v>
       </c>
       <c r="I47" s="17" t="str">
-        <v>⚠+920.5%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="48">
@@ -6433,13 +6433,13 @@
         <v>¥0.803/张</v>
       </c>
       <c r="G48" s="17" t="str">
-        <v>$0.012</v>
+        <v>—</v>
       </c>
       <c r="H48" s="17" t="str">
         <v>—</v>
       </c>
       <c r="I48" s="17" t="str">
-        <v>⚠+929.5%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="49">
@@ -6462,13 +6462,13 @@
         <v>¥1.335/张</v>
       </c>
       <c r="G49" s="17" t="str">
-        <v>$0.02</v>
+        <v>—</v>
       </c>
       <c r="H49" s="17" t="str">
         <v>—</v>
       </c>
       <c r="I49" s="17" t="str">
-        <v>⚠+926.9%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="50">
@@ -6491,13 +6491,13 @@
         <v>¥1.583/张</v>
       </c>
       <c r="G50" s="17" t="str">
-        <v>$0.006</v>
+        <v>—</v>
       </c>
       <c r="H50" s="17" t="str">
         <v>—</v>
       </c>
       <c r="I50" s="17" t="str">
-        <v>⚠+3959%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="51">
@@ -6520,13 +6520,13 @@
         <v>¥3.21/张</v>
       </c>
       <c r="G51" s="17" t="str">
-        <v>$0.012</v>
+        <v>—</v>
       </c>
       <c r="H51" s="17" t="str">
         <v>—</v>
       </c>
       <c r="I51" s="17" t="str">
-        <v>⚠+4015.4%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="52">
@@ -6549,13 +6549,13 @@
         <v>¥5.34/张</v>
       </c>
       <c r="G52" s="17" t="str">
-        <v>$0.02</v>
+        <v>—</v>
       </c>
       <c r="H52" s="17" t="str">
         <v>—</v>
       </c>
       <c r="I52" s="17" t="str">
-        <v>⚠+4007.7%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="53">
@@ -6578,13 +6578,13 @@
         <v>¥0.3/张</v>
       </c>
       <c r="G53" s="17" t="str">
-        <v>$0.006</v>
+        <v>—</v>
       </c>
       <c r="H53" s="17" t="str">
         <v>—</v>
       </c>
       <c r="I53" s="17" t="str">
-        <v>⚠+669.2%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="54">
@@ -6607,13 +6607,13 @@
         <v>¥0.338/张</v>
       </c>
       <c r="G54" s="17" t="str">
-        <v>$0.012</v>
+        <v>—</v>
       </c>
       <c r="H54" s="17" t="str">
         <v>—</v>
       </c>
       <c r="I54" s="17" t="str">
-        <v>⚠+333.3%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="55">
@@ -6636,13 +6636,13 @@
         <v>¥0.398/张</v>
       </c>
       <c r="G55" s="17" t="str">
-        <v>$0.02</v>
+        <v>—</v>
       </c>
       <c r="H55" s="17" t="str">
         <v>—</v>
       </c>
       <c r="I55" s="17" t="str">
-        <v>⚠+206.2%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="56">
@@ -6665,13 +6665,13 @@
         <v>¥0.638/张</v>
       </c>
       <c r="G56" s="17" t="str">
-        <v>$0.006</v>
+        <v>—</v>
       </c>
       <c r="H56" s="17" t="str">
         <v>—</v>
       </c>
       <c r="I56" s="17" t="str">
-        <v>⚠+1535.9%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="57">
@@ -6694,13 +6694,13 @@
         <v>¥1.05/张</v>
       </c>
       <c r="G57" s="17" t="str">
-        <v>$0.012</v>
+        <v>—</v>
       </c>
       <c r="H57" s="17" t="str">
         <v>—</v>
       </c>
       <c r="I57" s="17" t="str">
-        <v>⚠+1246.2%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="58">
@@ -6723,13 +6723,13 @@
         <v>¥1.583/张</v>
       </c>
       <c r="G58" s="17" t="str">
-        <v>$0.02</v>
+        <v>—</v>
       </c>
       <c r="H58" s="17" t="str">
         <v>—</v>
       </c>
       <c r="I58" s="17" t="str">
-        <v>⚠+1117.7%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="59">
@@ -6752,13 +6752,13 @@
         <v>¥1.838/张</v>
       </c>
       <c r="G59" s="17" t="str">
-        <v>$0.006</v>
+        <v>—</v>
       </c>
       <c r="H59" s="17" t="str">
         <v>—</v>
       </c>
       <c r="I59" s="17" t="str">
-        <v>⚠+4612.8%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="60">
@@ -6781,13 +6781,13 @@
         <v>¥3.45/张</v>
       </c>
       <c r="G60" s="17" t="str">
-        <v>$0.012</v>
+        <v>—</v>
       </c>
       <c r="H60" s="17" t="str">
         <v>—</v>
       </c>
       <c r="I60" s="17" t="str">
-        <v>⚠+4323.1%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="61">
@@ -6810,13 +6810,13 @@
         <v>¥5.588/张</v>
       </c>
       <c r="G61" s="17" t="str">
-        <v>$0.02</v>
+        <v>—</v>
       </c>
       <c r="H61" s="17" t="str">
         <v>—</v>
       </c>
       <c r="I61" s="17" t="str">
-        <v>⚠+4198.5%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="62">
@@ -7100,13 +7100,13 @@
         <v>¥0.1875/张</v>
       </c>
       <c r="G71" s="5" t="str">
-        <v>$0.0289</v>
+        <v>—</v>
       </c>
       <c r="H71" s="5" t="str">
         <v>✅ 一致</v>
       </c>
       <c r="I71" s="5" t="str">
-        <v>一致</v>
+        <v>—</v>
       </c>
     </row>
     <row r="72">
@@ -7129,13 +7129,13 @@
         <v>¥0.25/张</v>
       </c>
       <c r="G72" s="5" t="str">
-        <v>$0.0385</v>
+        <v>—</v>
       </c>
       <c r="H72" s="5" t="str">
         <v>✅ 一致</v>
       </c>
       <c r="I72" s="5" t="str">
-        <v>一致</v>
+        <v>—</v>
       </c>
     </row>
     <row r="73">
@@ -7158,13 +7158,13 @@
         <v>¥0.3125/张</v>
       </c>
       <c r="G73" s="5" t="str">
-        <v>$0.0481</v>
+        <v>—</v>
       </c>
       <c r="H73" s="5" t="str">
         <v>✅ 一致</v>
       </c>
       <c r="I73" s="5" t="str">
-        <v>一致</v>
+        <v>—</v>
       </c>
     </row>
     <row r="74">
@@ -7187,13 +7187,13 @@
         <v>¥0.25/张</v>
       </c>
       <c r="G74" s="5" t="str">
-        <v>$0.0289</v>
+        <v>—</v>
       </c>
       <c r="H74" s="5" t="str">
         <v>⚠+33.3%</v>
       </c>
       <c r="I74" s="5" t="str">
-        <v>⚠+33.1%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="75">
@@ -7216,13 +7216,13 @@
         <v>¥0.375/张</v>
       </c>
       <c r="G75" s="5" t="str">
-        <v>$0.0385</v>
+        <v>—</v>
       </c>
       <c r="H75" s="5" t="str">
         <v>⚠+50%</v>
       </c>
       <c r="I75" s="5" t="str">
-        <v>⚠+49.9%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="76">
@@ -7245,13 +7245,13 @@
         <v>¥0.5/张</v>
       </c>
       <c r="G76" s="5" t="str">
-        <v>$0.0481</v>
+        <v>—</v>
       </c>
       <c r="H76" s="5" t="str">
         <v>⚠+60%</v>
       </c>
       <c r="I76" s="5" t="str">
-        <v>⚠+59.9%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="77">
@@ -7274,13 +7274,13 @@
         <v>¥0.3125/张</v>
       </c>
       <c r="G77" s="5" t="str">
-        <v>$0.0289</v>
+        <v>—</v>
       </c>
       <c r="H77" s="5" t="str">
         <v>⚠+66.7%</v>
       </c>
       <c r="I77" s="5" t="str">
-        <v>⚠+66.4%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="78">
@@ -7303,13 +7303,13 @@
         <v>¥0.625/张</v>
       </c>
       <c r="G78" s="5" t="str">
-        <v>$0.0385</v>
+        <v>—</v>
       </c>
       <c r="H78" s="5" t="str">
         <v>⚠+150%</v>
       </c>
       <c r="I78" s="5" t="str">
-        <v>⚠+149.8%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="79">
@@ -7332,13 +7332,13 @@
         <v>¥0.9375/张</v>
       </c>
       <c r="G79" s="5" t="str">
-        <v>$0.0481</v>
+        <v>—</v>
       </c>
       <c r="H79" s="5" t="str">
         <v>⚠+200%</v>
       </c>
       <c r="I79" s="5" t="str">
-        <v>⚠+199.9%</v>
+        <v>—</v>
       </c>
     </row>
   </sheetData>
@@ -8564,13 +8564,13 @@
         <v>$0.0154/张</v>
       </c>
       <c r="G40" s="15" t="str">
-        <v>$0.006</v>
+        <v>—</v>
       </c>
       <c r="H40" s="15" t="str">
         <v>⚠+156.7%</v>
       </c>
       <c r="I40" s="15" t="str">
-        <v>⚠+156.7%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="41">
@@ -8593,13 +8593,13 @@
         <v>$0.006/张</v>
       </c>
       <c r="G41" s="15" t="str">
-        <v>$0.006</v>
+        <v>—</v>
       </c>
       <c r="H41" s="15" t="str">
         <v>✅ 一致</v>
       </c>
       <c r="I41" s="15" t="str">
-        <v>一致</v>
+        <v>—</v>
       </c>
     </row>
     <row r="42">
@@ -8622,13 +8622,13 @@
         <v>$0.012/张</v>
       </c>
       <c r="G42" s="15" t="str">
-        <v>$0.012</v>
+        <v>—</v>
       </c>
       <c r="H42" s="15" t="str">
         <v>✅ 一致</v>
       </c>
       <c r="I42" s="15" t="str">
-        <v>一致</v>
+        <v>—</v>
       </c>
     </row>
     <row r="43">
@@ -8651,13 +8651,13 @@
         <v>$0.02/张</v>
       </c>
       <c r="G43" s="15" t="str">
-        <v>$0.02</v>
+        <v>—</v>
       </c>
       <c r="H43" s="15" t="str">
         <v>✅ 一致</v>
       </c>
       <c r="I43" s="15" t="str">
-        <v>一致</v>
+        <v>—</v>
       </c>
     </row>
     <row r="44">
@@ -8680,13 +8680,13 @@
         <v>$0.053/张</v>
       </c>
       <c r="G44" s="15" t="str">
-        <v>$0.006</v>
+        <v>—</v>
       </c>
       <c r="H44" s="15" t="str">
         <v>⚠+783.3%</v>
       </c>
       <c r="I44" s="15" t="str">
-        <v>⚠+783.3%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="45">
@@ -8709,13 +8709,13 @@
         <v>$0.107/张</v>
       </c>
       <c r="G45" s="15" t="str">
-        <v>$0.012</v>
+        <v>—</v>
       </c>
       <c r="H45" s="15" t="str">
         <v>⚠+791.7%</v>
       </c>
       <c r="I45" s="15" t="str">
-        <v>⚠+791.7%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="46">
@@ -8738,13 +8738,13 @@
         <v>$0.178/张</v>
       </c>
       <c r="G46" s="15" t="str">
-        <v>$0.02</v>
+        <v>—</v>
       </c>
       <c r="H46" s="15" t="str">
         <v>⚠+790%</v>
       </c>
       <c r="I46" s="15" t="str">
-        <v>⚠+790%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="47">
@@ -8767,13 +8767,13 @@
         <v>$0.211/张</v>
       </c>
       <c r="G47" s="15" t="str">
-        <v>$0.006</v>
+        <v>—</v>
       </c>
       <c r="H47" s="15" t="str">
         <v>⚠+3416.7%</v>
       </c>
       <c r="I47" s="15" t="str">
-        <v>⚠+3416.7%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="48">
@@ -8796,13 +8796,13 @@
         <v>$0.428/张</v>
       </c>
       <c r="G48" s="15" t="str">
-        <v>$0.012</v>
+        <v>—</v>
       </c>
       <c r="H48" s="15" t="str">
         <v>⚠+3466.7%</v>
       </c>
       <c r="I48" s="15" t="str">
-        <v>⚠+3466.7%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="49">
@@ -8825,13 +8825,13 @@
         <v>$0.712/张</v>
       </c>
       <c r="G49" s="15" t="str">
-        <v>$0.02</v>
+        <v>—</v>
       </c>
       <c r="H49" s="15" t="str">
         <v>⚠+3460%</v>
       </c>
       <c r="I49" s="15" t="str">
-        <v>⚠+3460%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="50">
@@ -8854,13 +8854,13 @@
         <v>$0.04/张</v>
       </c>
       <c r="G50" s="15" t="str">
-        <v>$0.006</v>
+        <v>—</v>
       </c>
       <c r="H50" s="15" t="str">
         <v>⚠+566.7%</v>
       </c>
       <c r="I50" s="15" t="str">
-        <v>⚠+566.7%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="51">
@@ -8883,13 +8883,13 @@
         <v>$0.045/张</v>
       </c>
       <c r="G51" s="15" t="str">
-        <v>$0.012</v>
+        <v>—</v>
       </c>
       <c r="H51" s="15" t="str">
         <v>⚠+275%</v>
       </c>
       <c r="I51" s="15" t="str">
-        <v>⚠+275%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="52">
@@ -8912,13 +8912,13 @@
         <v>$0.053/张</v>
       </c>
       <c r="G52" s="15" t="str">
-        <v>$0.02</v>
+        <v>—</v>
       </c>
       <c r="H52" s="15" t="str">
         <v>⚠+165%</v>
       </c>
       <c r="I52" s="15" t="str">
-        <v>⚠+165%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="53">
@@ -8941,13 +8941,13 @@
         <v>$0.085/张</v>
       </c>
       <c r="G53" s="15" t="str">
-        <v>$0.006</v>
+        <v>—</v>
       </c>
       <c r="H53" s="15" t="str">
         <v>⚠+1316.7%</v>
       </c>
       <c r="I53" s="15" t="str">
-        <v>⚠+1316.7%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="54">
@@ -8970,13 +8970,13 @@
         <v>$0.14/张</v>
       </c>
       <c r="G54" s="15" t="str">
-        <v>$0.012</v>
+        <v>—</v>
       </c>
       <c r="H54" s="15" t="str">
         <v>⚠+1066.7%</v>
       </c>
       <c r="I54" s="15" t="str">
-        <v>⚠+1066.7%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="55">
@@ -8999,13 +8999,13 @@
         <v>$0.211/张</v>
       </c>
       <c r="G55" s="15" t="str">
-        <v>$0.02</v>
+        <v>—</v>
       </c>
       <c r="H55" s="15" t="str">
         <v>⚠+955%</v>
       </c>
       <c r="I55" s="15" t="str">
-        <v>⚠+955%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="56">
@@ -9028,13 +9028,13 @@
         <v>$0.245/张</v>
       </c>
       <c r="G56" s="15" t="str">
-        <v>$0.006</v>
+        <v>—</v>
       </c>
       <c r="H56" s="15" t="str">
         <v>⚠+3983.3%</v>
       </c>
       <c r="I56" s="15" t="str">
-        <v>⚠+3983.3%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="57">
@@ -9057,13 +9057,13 @@
         <v>$0.46/张</v>
       </c>
       <c r="G57" s="15" t="str">
-        <v>$0.012</v>
+        <v>—</v>
       </c>
       <c r="H57" s="15" t="str">
         <v>⚠+3733.3%</v>
       </c>
       <c r="I57" s="15" t="str">
-        <v>⚠+3733.3%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="58">
@@ -9086,13 +9086,13 @@
         <v>$0.745/张</v>
       </c>
       <c r="G58" s="15" t="str">
-        <v>$0.02</v>
+        <v>—</v>
       </c>
       <c r="H58" s="15" t="str">
         <v>⚠+3625%</v>
       </c>
       <c r="I58" s="15" t="str">
-        <v>⚠+3625%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="59">
@@ -9376,13 +9376,13 @@
         <v>$0.0288461538461539/张</v>
       </c>
       <c r="G68" s="19" t="str">
-        <v>$0.0289</v>
+        <v>—</v>
       </c>
       <c r="H68" s="19" t="str">
         <v>✅ 一致</v>
       </c>
       <c r="I68" s="19" t="str">
-        <v>一致</v>
+        <v>—</v>
       </c>
     </row>
     <row r="69">
@@ -9405,13 +9405,13 @@
         <v>$0.0384615384615385/张</v>
       </c>
       <c r="G69" s="19" t="str">
-        <v>$0.0385</v>
+        <v>—</v>
       </c>
       <c r="H69" s="19" t="str">
         <v>✅ 一致</v>
       </c>
       <c r="I69" s="19" t="str">
-        <v>一致</v>
+        <v>—</v>
       </c>
     </row>
     <row r="70">
@@ -9434,13 +9434,13 @@
         <v>$0.0480769230769231/张</v>
       </c>
       <c r="G70" s="19" t="str">
-        <v>$0.0481</v>
+        <v>—</v>
       </c>
       <c r="H70" s="19" t="str">
         <v>✅ 一致</v>
       </c>
       <c r="I70" s="19" t="str">
-        <v>一致</v>
+        <v>—</v>
       </c>
     </row>
     <row r="71">
@@ -9463,13 +9463,13 @@
         <v>$0.0384615384615385/张</v>
       </c>
       <c r="G71" s="19" t="str">
-        <v>$0.0289</v>
+        <v>—</v>
       </c>
       <c r="H71" s="19" t="str">
         <v>⚠+33.3%</v>
       </c>
       <c r="I71" s="19" t="str">
-        <v>⚠+33.1%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="72">
@@ -9492,13 +9492,13 @@
         <v>$0.0576923076923077/张</v>
       </c>
       <c r="G72" s="19" t="str">
-        <v>$0.0385</v>
+        <v>—</v>
       </c>
       <c r="H72" s="19" t="str">
         <v>⚠+50%</v>
       </c>
       <c r="I72" s="19" t="str">
-        <v>⚠+49.9%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="73">
@@ -9521,13 +9521,13 @@
         <v>$0.0769230769230769/张</v>
       </c>
       <c r="G73" s="19" t="str">
-        <v>$0.0481</v>
+        <v>—</v>
       </c>
       <c r="H73" s="19" t="str">
         <v>⚠+60%</v>
       </c>
       <c r="I73" s="19" t="str">
-        <v>⚠+59.9%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="74">
@@ -9550,13 +9550,13 @@
         <v>$0.0480769230769231/张</v>
       </c>
       <c r="G74" s="19" t="str">
-        <v>$0.0289</v>
+        <v>—</v>
       </c>
       <c r="H74" s="19" t="str">
         <v>⚠+66.7%</v>
       </c>
       <c r="I74" s="19" t="str">
-        <v>⚠+66.4%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="75">
@@ -9579,13 +9579,13 @@
         <v>$0.0961538461538462/张</v>
       </c>
       <c r="G75" s="19" t="str">
-        <v>$0.0385</v>
+        <v>—</v>
       </c>
       <c r="H75" s="19" t="str">
         <v>⚠+150%</v>
       </c>
       <c r="I75" s="19" t="str">
-        <v>⚠+149.8%</v>
+        <v>—</v>
       </c>
     </row>
     <row r="76">
@@ -9608,13 +9608,13 @@
         <v>$0.144230769230769/张</v>
       </c>
       <c r="G76" s="19" t="str">
-        <v>$0.0481</v>
+        <v>—</v>
       </c>
       <c r="H76" s="19" t="str">
         <v>⚠+200%</v>
       </c>
       <c r="I76" s="19" t="str">
-        <v>⚠+199.9%</v>
+        <v>—</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(pricing): treat Kling image API capability tiers as official coverage
Use klingai.com document-api image pricing as the seed source, and alert when Trinity listing misses official capability×resolution slots such as Kling-2.1 image-to-image.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/pricing/output/trinity-pricing-image.xlsx
+++ b/pricing/output/trinity-pricing-image.xlsx
@@ -560,10 +560,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -595,10 +595,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -2497,7 +2497,7 @@
         <v>价✅</v>
       </c>
       <c r="Q31" s="16" t="str">
-        <v>灵感值/Credits 计价，无公开按张 API 价目</v>
+        <v>开放平台 API 价目：能力分档（文生图/图生图/多图参考）</v>
       </c>
     </row>
     <row r="32">
@@ -2550,7 +2550,7 @@
         <v>价✅</v>
       </c>
       <c r="Q32" s="15" t="str">
-        <v>灵感值/Credits 计价，无公开按张 API 价目</v>
+        <v>开放平台 API 价目：能力分档（文生图/图生图/多图参考）</v>
       </c>
     </row>
     <row r="33">
@@ -2570,7 +2570,7 @@
         <v>4K</v>
       </c>
       <c r="F33" s="15" t="str">
-        <v>¥0.26/张</v>
+        <v>—</v>
       </c>
       <c r="G33" s="15" t="str">
         <v>¥0.26/张</v>
@@ -2588,10 +2588,10 @@
         <v>—</v>
       </c>
       <c r="L33" s="15" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="M33" s="15" t="str">
-        <v>⚠-7.5%</v>
+        <v>—</v>
       </c>
       <c r="N33" s="15" t="str">
         <v>—</v>
@@ -2603,7 +2603,7 @@
         <v>ℹ 线上无同档刊例</v>
       </c>
       <c r="Q33" s="15" t="str">
-        <v>灵感值/Credits 计价，无公开按张 API 价目</v>
+        <v>开放平台 API 价目：能力分档（文生图/图生图/多图参考）</v>
       </c>
     </row>
     <row r="34">
@@ -2656,7 +2656,7 @@
         <v>价✅</v>
       </c>
       <c r="Q34" s="15" t="str">
-        <v>灵感值/Credits 计价，无公开按张 API 价目</v>
+        <v>开放平台 API 价目：能力分档（文生图/图生图/多图参考）</v>
       </c>
     </row>
     <row r="35">
@@ -2709,7 +2709,7 @@
         <v>价✅</v>
       </c>
       <c r="Q35" s="15" t="str">
-        <v>灵感值/Credits 计价，无公开按张 API 价目</v>
+        <v>开放平台 API 价目：能力分档（文生图/图生图/多图参考）</v>
       </c>
     </row>
     <row r="36">
@@ -2729,7 +2729,7 @@
         <v>4K</v>
       </c>
       <c r="F36" s="15" t="str">
-        <v>¥0.4/张</v>
+        <v>—</v>
       </c>
       <c r="G36" s="15" t="str">
         <v>¥0.4/张</v>
@@ -2747,10 +2747,10 @@
         <v>$0.0616/张</v>
       </c>
       <c r="L36" s="15" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="M36" s="15" t="str">
-        <v>⚠-9%</v>
+        <v>—</v>
       </c>
       <c r="N36" s="15" t="str">
         <v>—</v>
@@ -2759,10 +2759,10 @@
         <v>—</v>
       </c>
       <c r="P36" s="15" t="str">
-        <v>价✅</v>
+        <v>ℹ 官方无档 · 价⚠+10%</v>
       </c>
       <c r="Q36" s="15" t="str">
-        <v>灵感值/Credits 计价，无公开按张 API 价目</v>
+        <v>开放平台 API 价目：能力分档（文生图/图生图/多图参考）</v>
       </c>
     </row>
     <row r="37">
@@ -2815,7 +2815,7 @@
         <v>价✅</v>
       </c>
       <c r="Q37" s="15" t="str">
-        <v>灵感值/Credits 计价，无公开按张 API 价目</v>
+        <v>开放平台 API 价目：能力分档（文生图/图生图/多图参考）</v>
       </c>
     </row>
     <row r="38">
@@ -2868,7 +2868,7 @@
         <v>价✅</v>
       </c>
       <c r="Q38" s="15" t="str">
-        <v>灵感值/Credits 计价，无公开按张 API 价目</v>
+        <v>开放平台 API 价目：能力分档（文生图/图生图/多图参考）</v>
       </c>
     </row>
     <row r="39">
@@ -2921,7 +2921,7 @@
         <v>价✅</v>
       </c>
       <c r="Q39" s="15" t="str">
-        <v>灵感值/Credits 计价，无公开按张 API 价目</v>
+        <v>开放平台 API 价目：能力分档（文生图/图生图/多图参考）</v>
       </c>
     </row>
     <row r="40">
@@ -2974,7 +2974,7 @@
         <v>价✅</v>
       </c>
       <c r="Q40" s="15" t="str">
-        <v>灵感值/Credits 计价，无公开按张 API 价目</v>
+        <v>开放平台 API 价目：能力分档（文生图/图生图/多图参考）</v>
       </c>
     </row>
     <row r="41">
@@ -3027,7 +3027,7 @@
         <v>价✅</v>
       </c>
       <c r="Q41" s="15" t="str">
-        <v>灵感值/Credits 计价，无公开按张 API 价目</v>
+        <v>开放平台 API 价目：能力分档（文生图/图生图/多图参考）</v>
       </c>
     </row>
     <row r="42">
@@ -3047,7 +3047,7 @@
         <v>4K</v>
       </c>
       <c r="F42" s="15" t="str">
-        <v>¥0.4/张</v>
+        <v>—</v>
       </c>
       <c r="G42" s="15" t="str">
         <v>¥0.4/张</v>
@@ -3065,10 +3065,10 @@
         <v>$0.0616/张</v>
       </c>
       <c r="L42" s="15" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="M42" s="15" t="str">
-        <v>⚠-9%</v>
+        <v>—</v>
       </c>
       <c r="N42" s="15" t="str">
         <v>—</v>
@@ -3077,10 +3077,10 @@
         <v>—</v>
       </c>
       <c r="P42" s="15" t="str">
-        <v>价✅</v>
+        <v>ℹ 官方无档 · 价⚠+10%</v>
       </c>
       <c r="Q42" s="15" t="str">
-        <v>灵感值/Credits 计价，无公开按张 API 价目</v>
+        <v>开放平台 API 价目：能力分档（文生图/图生图/多图参考）</v>
       </c>
     </row>
     <row r="43">
@@ -4173,7 +4173,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K36"/>
   <cols>
     <col min="1" max="1" width="56.83203125" customWidth="1"/>
     <col min="2" max="2" width="13.83203125" customWidth="1"/>
@@ -4183,9 +4183,9 @@
     <col min="6" max="6" width="14.83203125" customWidth="1"/>
     <col min="7" max="7" width="11.83203125" customWidth="1"/>
     <col min="8" max="8" width="13.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="17.83203125" customWidth="1"/>
     <col min="10" max="10" width="13.83203125" customWidth="1"/>
-    <col min="11" max="11" width="48.83203125" customWidth="1"/>
+    <col min="11" max="11" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4231,10 +4231,10 @@
         <v>18</v>
       </c>
       <c r="C2" s="21">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D2" s="21">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E2" s="21">
         <v>7</v>
@@ -4243,19 +4243,19 @@
         <v>55</v>
       </c>
       <c r="G2" s="21">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="H2" s="21">
+        <v>8</v>
+      </c>
+      <c r="I2" s="21" t="str">
+        <v>+20% ~ +160%</v>
+      </c>
+      <c r="J2" s="21">
         <v>5</v>
       </c>
-      <c r="I2" s="21" t="str">
-        <v>+20% ~ +84%</v>
-      </c>
-      <c r="J2" s="21">
-        <v>2</v>
-      </c>
       <c r="K2" s="21" t="str">
-        <v>Hunyuan-3.0(+80%)；qwen-0925(+84%)</v>
+        <v>Hunyuan-3.0(+80%)；qwen-0925(+84%)；Kling-3.0(+100%)；Kling-O1(+100%)；Kling-2.1(+160%)</v>
       </c>
     </row>
     <row r="3">
@@ -4284,13 +4284,13 @@
         <v>21</v>
       </c>
       <c r="I3" s="21" t="str">
-        <v>+0.7% ~ +84%</v>
+        <v>+0.7% ~ +140.5%</v>
       </c>
       <c r="J3" s="21">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K3" s="21" t="str">
-        <v>qwen-0925(+84%)；MJ-v7(+61.5%)；GG-2.5(+61.5%)</v>
+        <v>qwen-0925(+84%)；MJ-v7(+61.5%)；GG-2.5(+61.5%)；Kling-3.0(+82%)；Kling-O1(+82%)；Kling-2.1(+140.5%)</v>
       </c>
     </row>
     <row r="4">
@@ -4575,22 +4575,22 @@
     </row>
     <row r="12">
       <c r="A12" s="21" t="str">
-        <v>AIGC国际站-生图</v>
+        <v>AIGC国内站-生图</v>
       </c>
       <c r="B12" s="21" t="str">
-        <v>qwen-0925</v>
+        <v>Kling-3.0</v>
       </c>
       <c r="C12" s="21" t="str">
-        <v>通义 0925</v>
+        <v>可灵 3</v>
       </c>
       <c r="D12" s="21" t="str">
-        <v>标准价·1K</v>
+        <v>标准价·4K</v>
       </c>
       <c r="E12" s="21" t="str">
-        <v>+20%</v>
+        <v>+100%</v>
       </c>
       <c r="F12" s="21" t="str">
-        <v>⚠+20%</v>
+        <v>⚠+100%</v>
       </c>
       <c r="G12" s="21" t="str">
         <v/>
@@ -4610,22 +4610,22 @@
     </row>
     <row r="13">
       <c r="A13" s="21" t="str">
-        <v/>
+        <v>AIGC国内站-生图</v>
       </c>
       <c r="B13" s="21" t="str">
-        <v/>
+        <v>Kling-O1</v>
       </c>
       <c r="C13" s="21" t="str">
-        <v/>
+        <v>可灵 O1</v>
       </c>
       <c r="D13" s="21" t="str">
-        <v>标准价·2K</v>
+        <v>标准价·4K</v>
       </c>
       <c r="E13" s="21" t="str">
-        <v>+52%</v>
+        <v>+100%</v>
       </c>
       <c r="F13" s="21" t="str">
-        <v>⚠+52%</v>
+        <v>⚠+100%</v>
       </c>
       <c r="G13" s="21" t="str">
         <v/>
@@ -4645,22 +4645,22 @@
     </row>
     <row r="14">
       <c r="A14" s="21" t="str">
-        <v/>
+        <v>AIGC国内站-生图</v>
       </c>
       <c r="B14" s="21" t="str">
-        <v/>
+        <v>Kling-2.1</v>
       </c>
       <c r="C14" s="21" t="str">
-        <v/>
+        <v>可灵 2.1</v>
       </c>
       <c r="D14" s="21" t="str">
-        <v>标准价·4K</v>
+        <v>文生图·4K</v>
       </c>
       <c r="E14" s="21" t="str">
-        <v>+84%</v>
+        <v>+160%</v>
       </c>
       <c r="F14" s="21" t="str">
-        <v>⚠+84%</v>
+        <v>⚠+160%</v>
       </c>
       <c r="G14" s="21" t="str">
         <v/>
@@ -4683,19 +4683,19 @@
         <v>AIGC国际站-生图</v>
       </c>
       <c r="B15" s="21" t="str">
-        <v>MJ-v7</v>
+        <v>qwen-0925</v>
       </c>
       <c r="C15" s="21" t="str">
-        <v>Midjourney v7</v>
+        <v>通义 0925</v>
       </c>
       <c r="D15" s="21" t="str">
-        <v>标准价·2K</v>
+        <v>标准价·1K</v>
       </c>
       <c r="E15" s="21" t="str">
-        <v>+30.8%</v>
+        <v>+20%</v>
       </c>
       <c r="F15" s="21" t="str">
-        <v>⚠+30.8%</v>
+        <v>⚠+20%</v>
       </c>
       <c r="G15" s="21" t="str">
         <v/>
@@ -4724,13 +4724,13 @@
         <v/>
       </c>
       <c r="D16" s="21" t="str">
-        <v>标准价·4K</v>
+        <v>标准价·2K</v>
       </c>
       <c r="E16" s="21" t="str">
-        <v>+61.5%</v>
+        <v>+52%</v>
       </c>
       <c r="F16" s="21" t="str">
-        <v>⚠+61.5%</v>
+        <v>⚠+52%</v>
       </c>
       <c r="G16" s="21" t="str">
         <v/>
@@ -4750,22 +4750,22 @@
     </row>
     <row r="17">
       <c r="A17" s="21" t="str">
-        <v>AIGC国际站-生图</v>
+        <v/>
       </c>
       <c r="B17" s="21" t="str">
-        <v>GG-2.5</v>
+        <v/>
       </c>
       <c r="C17" s="21" t="str">
-        <v>Gemini 2.5（超分暂时按1K收）</v>
+        <v/>
       </c>
       <c r="D17" s="21" t="str">
-        <v>是·2K</v>
+        <v>标准价·4K</v>
       </c>
       <c r="E17" s="21" t="str">
-        <v>+30.8%</v>
+        <v>+84%</v>
       </c>
       <c r="F17" s="21" t="str">
-        <v>⚠+30.8%</v>
+        <v>⚠+84%</v>
       </c>
       <c r="G17" s="21" t="str">
         <v/>
@@ -4785,22 +4785,22 @@
     </row>
     <row r="18">
       <c r="A18" s="21" t="str">
-        <v/>
+        <v>AIGC国际站-生图</v>
       </c>
       <c r="B18" s="21" t="str">
-        <v/>
+        <v>MJ-v7</v>
       </c>
       <c r="C18" s="21" t="str">
-        <v/>
+        <v>Midjourney v7</v>
       </c>
       <c r="D18" s="21" t="str">
-        <v>是·4K</v>
+        <v>标准价·2K</v>
       </c>
       <c r="E18" s="21" t="str">
-        <v>+61.5%</v>
+        <v>+30.8%</v>
       </c>
       <c r="F18" s="21" t="str">
-        <v>⚠+61.5%</v>
+        <v>⚠+30.8%</v>
       </c>
       <c r="G18" s="21" t="str">
         <v/>
@@ -4829,13 +4829,13 @@
         <v/>
       </c>
       <c r="D19" s="21" t="str">
-        <v/>
+        <v>标准价·4K</v>
       </c>
       <c r="E19" s="21" t="str">
-        <v/>
+        <v>+61.5%</v>
       </c>
       <c r="F19" s="21" t="str">
-        <v/>
+        <v>⚠+61.5%</v>
       </c>
       <c r="G19" s="21" t="str">
         <v/>
@@ -4855,22 +4855,22 @@
     </row>
     <row r="20">
       <c r="A20" s="21" t="str">
-        <v>—— 偏差≥50% · 待核验（未登记例外）——</v>
+        <v>AIGC国际站-生图</v>
       </c>
       <c r="B20" s="21" t="str">
-        <v/>
+        <v>GG-2.5</v>
       </c>
       <c r="C20" s="21" t="str">
-        <v/>
+        <v>Gemini 2.5（超分暂时按1K收）</v>
       </c>
       <c r="D20" s="21" t="str">
-        <v/>
+        <v>是·2K</v>
       </c>
       <c r="E20" s="21" t="str">
-        <v/>
+        <v>+30.8%</v>
       </c>
       <c r="F20" s="21" t="str">
-        <v/>
+        <v>⚠+30.8%</v>
       </c>
       <c r="G20" s="21" t="str">
         <v/>
@@ -4890,22 +4890,22 @@
     </row>
     <row r="21">
       <c r="A21" s="21" t="str">
-        <v>供应商</v>
+        <v/>
       </c>
       <c r="B21" s="21" t="str">
-        <v>Trinity ID</v>
+        <v/>
       </c>
       <c r="C21" s="21" t="str">
-        <v>显示名</v>
+        <v/>
       </c>
       <c r="D21" s="21" t="str">
-        <v>档位</v>
+        <v>是·4K</v>
       </c>
       <c r="E21" s="21" t="str">
-        <v>偏差%</v>
+        <v>+61.5%</v>
       </c>
       <c r="F21" s="21" t="str">
-        <v>供应商vs官方</v>
+        <v>⚠+61.5%</v>
       </c>
       <c r="G21" s="21" t="str">
         <v/>
@@ -4925,22 +4925,22 @@
     </row>
     <row r="22">
       <c r="A22" s="21" t="str">
-        <v/>
+        <v>AIGC国际站-生图</v>
       </c>
       <c r="B22" s="21" t="str">
-        <v/>
+        <v>Kling-3.0</v>
       </c>
       <c r="C22" s="21" t="str">
-        <v/>
+        <v>可灵 3</v>
       </c>
       <c r="D22" s="21" t="str">
-        <v/>
+        <v>标准价·1K</v>
       </c>
       <c r="E22" s="21" t="str">
-        <v/>
+        <v>+9%</v>
       </c>
       <c r="F22" s="21" t="str">
-        <v/>
+        <v>⚠-9%</v>
       </c>
       <c r="G22" s="21" t="str">
         <v/>
@@ -4960,7 +4960,7 @@
     </row>
     <row r="23">
       <c r="A23" s="21" t="str">
-        <v>生成时间：2026-08-18T07:48:14Z</v>
+        <v/>
       </c>
       <c r="B23" s="21" t="str">
         <v/>
@@ -4969,13 +4969,13 @@
         <v/>
       </c>
       <c r="D23" s="21" t="str">
-        <v/>
+        <v>标准价·2K</v>
       </c>
       <c r="E23" s="21" t="str">
-        <v/>
+        <v>+9%</v>
       </c>
       <c r="F23" s="21" t="str">
-        <v/>
+        <v>⚠-9%</v>
       </c>
       <c r="G23" s="21" t="str">
         <v/>
@@ -4995,42 +4995,462 @@
     </row>
     <row r="24">
       <c r="A24" s="21" t="str">
+        <v/>
+      </c>
+      <c r="B24" s="21" t="str">
+        <v/>
+      </c>
+      <c r="C24" s="21" t="str">
+        <v/>
+      </c>
+      <c r="D24" s="21" t="str">
+        <v>标准价·4K</v>
+      </c>
+      <c r="E24" s="21" t="str">
+        <v>+82%</v>
+      </c>
+      <c r="F24" s="21" t="str">
+        <v>⚠+82%</v>
+      </c>
+      <c r="G24" s="21" t="str">
+        <v/>
+      </c>
+      <c r="H24" s="21" t="str">
+        <v/>
+      </c>
+      <c r="I24" s="21" t="str">
+        <v/>
+      </c>
+      <c r="J24" s="21" t="str">
+        <v/>
+      </c>
+      <c r="K24" s="21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="21" t="str">
+        <v>AIGC国际站-生图</v>
+      </c>
+      <c r="B25" s="21" t="str">
+        <v>Kling-O1</v>
+      </c>
+      <c r="C25" s="21" t="str">
+        <v>可灵 O1</v>
+      </c>
+      <c r="D25" s="21" t="str">
+        <v>标准价·1K</v>
+      </c>
+      <c r="E25" s="21" t="str">
+        <v>+9%</v>
+      </c>
+      <c r="F25" s="21" t="str">
+        <v>⚠-9%</v>
+      </c>
+      <c r="G25" s="21" t="str">
+        <v/>
+      </c>
+      <c r="H25" s="21" t="str">
+        <v/>
+      </c>
+      <c r="I25" s="21" t="str">
+        <v/>
+      </c>
+      <c r="J25" s="21" t="str">
+        <v/>
+      </c>
+      <c r="K25" s="21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="21" t="str">
+        <v/>
+      </c>
+      <c r="B26" s="21" t="str">
+        <v/>
+      </c>
+      <c r="C26" s="21" t="str">
+        <v/>
+      </c>
+      <c r="D26" s="21" t="str">
+        <v>标准价·2K</v>
+      </c>
+      <c r="E26" s="21" t="str">
+        <v>+9%</v>
+      </c>
+      <c r="F26" s="21" t="str">
+        <v>⚠-9%</v>
+      </c>
+      <c r="G26" s="21" t="str">
+        <v/>
+      </c>
+      <c r="H26" s="21" t="str">
+        <v/>
+      </c>
+      <c r="I26" s="21" t="str">
+        <v/>
+      </c>
+      <c r="J26" s="21" t="str">
+        <v/>
+      </c>
+      <c r="K26" s="21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="21" t="str">
+        <v/>
+      </c>
+      <c r="B27" s="21" t="str">
+        <v/>
+      </c>
+      <c r="C27" s="21" t="str">
+        <v/>
+      </c>
+      <c r="D27" s="21" t="str">
+        <v>标准价·4K</v>
+      </c>
+      <c r="E27" s="21" t="str">
+        <v>+82%</v>
+      </c>
+      <c r="F27" s="21" t="str">
+        <v>⚠+82%</v>
+      </c>
+      <c r="G27" s="21" t="str">
+        <v/>
+      </c>
+      <c r="H27" s="21" t="str">
+        <v/>
+      </c>
+      <c r="I27" s="21" t="str">
+        <v/>
+      </c>
+      <c r="J27" s="21" t="str">
+        <v/>
+      </c>
+      <c r="K27" s="21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="21" t="str">
+        <v>AIGC国际站-生图</v>
+      </c>
+      <c r="B28" s="21" t="str">
+        <v>Kling-2.1</v>
+      </c>
+      <c r="C28" s="21" t="str">
+        <v>可灵 2.1</v>
+      </c>
+      <c r="D28" s="21" t="str">
+        <v>文生图·1K</v>
+      </c>
+      <c r="E28" s="21" t="str">
+        <v>+9%</v>
+      </c>
+      <c r="F28" s="21" t="str">
+        <v>⚠-9%</v>
+      </c>
+      <c r="G28" s="21" t="str">
+        <v/>
+      </c>
+      <c r="H28" s="21" t="str">
+        <v/>
+      </c>
+      <c r="I28" s="21" t="str">
+        <v/>
+      </c>
+      <c r="J28" s="21" t="str">
+        <v/>
+      </c>
+      <c r="K28" s="21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="21" t="str">
+        <v/>
+      </c>
+      <c r="B29" s="21" t="str">
+        <v/>
+      </c>
+      <c r="C29" s="21" t="str">
+        <v/>
+      </c>
+      <c r="D29" s="21" t="str">
+        <v>文生图·2K</v>
+      </c>
+      <c r="E29" s="21" t="str">
+        <v>+9%</v>
+      </c>
+      <c r="F29" s="21" t="str">
+        <v>⚠-9%</v>
+      </c>
+      <c r="G29" s="21" t="str">
+        <v/>
+      </c>
+      <c r="H29" s="21" t="str">
+        <v/>
+      </c>
+      <c r="I29" s="21" t="str">
+        <v/>
+      </c>
+      <c r="J29" s="21" t="str">
+        <v/>
+      </c>
+      <c r="K29" s="21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="21" t="str">
+        <v/>
+      </c>
+      <c r="B30" s="21" t="str">
+        <v/>
+      </c>
+      <c r="C30" s="21" t="str">
+        <v/>
+      </c>
+      <c r="D30" s="21" t="str">
+        <v>文生图·4K</v>
+      </c>
+      <c r="E30" s="21" t="str">
+        <v>+140.5%</v>
+      </c>
+      <c r="F30" s="21" t="str">
+        <v>⚠+140.5%</v>
+      </c>
+      <c r="G30" s="21" t="str">
+        <v/>
+      </c>
+      <c r="H30" s="21" t="str">
+        <v/>
+      </c>
+      <c r="I30" s="21" t="str">
+        <v/>
+      </c>
+      <c r="J30" s="21" t="str">
+        <v/>
+      </c>
+      <c r="K30" s="21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="21" t="str">
+        <v/>
+      </c>
+      <c r="B31" s="21" t="str">
+        <v/>
+      </c>
+      <c r="C31" s="21" t="str">
+        <v/>
+      </c>
+      <c r="D31" s="21" t="str">
+        <v/>
+      </c>
+      <c r="E31" s="21" t="str">
+        <v/>
+      </c>
+      <c r="F31" s="21" t="str">
+        <v/>
+      </c>
+      <c r="G31" s="21" t="str">
+        <v/>
+      </c>
+      <c r="H31" s="21" t="str">
+        <v/>
+      </c>
+      <c r="I31" s="21" t="str">
+        <v/>
+      </c>
+      <c r="J31" s="21" t="str">
+        <v/>
+      </c>
+      <c r="K31" s="21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="21" t="str">
+        <v>—— 偏差≥50% · 待核验（未登记例外）——</v>
+      </c>
+      <c r="B32" s="21" t="str">
+        <v/>
+      </c>
+      <c r="C32" s="21" t="str">
+        <v/>
+      </c>
+      <c r="D32" s="21" t="str">
+        <v/>
+      </c>
+      <c r="E32" s="21" t="str">
+        <v/>
+      </c>
+      <c r="F32" s="21" t="str">
+        <v/>
+      </c>
+      <c r="G32" s="21" t="str">
+        <v/>
+      </c>
+      <c r="H32" s="21" t="str">
+        <v/>
+      </c>
+      <c r="I32" s="21" t="str">
+        <v/>
+      </c>
+      <c r="J32" s="21" t="str">
+        <v/>
+      </c>
+      <c r="K32" s="21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="21" t="str">
+        <v>供应商</v>
+      </c>
+      <c r="B33" s="21" t="str">
+        <v>Trinity ID</v>
+      </c>
+      <c r="C33" s="21" t="str">
+        <v>显示名</v>
+      </c>
+      <c r="D33" s="21" t="str">
+        <v>档位</v>
+      </c>
+      <c r="E33" s="21" t="str">
+        <v>偏差%</v>
+      </c>
+      <c r="F33" s="21" t="str">
+        <v>供应商vs官方</v>
+      </c>
+      <c r="G33" s="21" t="str">
+        <v/>
+      </c>
+      <c r="H33" s="21" t="str">
+        <v/>
+      </c>
+      <c r="I33" s="21" t="str">
+        <v/>
+      </c>
+      <c r="J33" s="21" t="str">
+        <v/>
+      </c>
+      <c r="K33" s="21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="21" t="str">
+        <v/>
+      </c>
+      <c r="B34" s="21" t="str">
+        <v/>
+      </c>
+      <c r="C34" s="21" t="str">
+        <v/>
+      </c>
+      <c r="D34" s="21" t="str">
+        <v/>
+      </c>
+      <c r="E34" s="21" t="str">
+        <v/>
+      </c>
+      <c r="F34" s="21" t="str">
+        <v/>
+      </c>
+      <c r="G34" s="21" t="str">
+        <v/>
+      </c>
+      <c r="H34" s="21" t="str">
+        <v/>
+      </c>
+      <c r="I34" s="21" t="str">
+        <v/>
+      </c>
+      <c r="J34" s="21" t="str">
+        <v/>
+      </c>
+      <c r="K34" s="21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="21" t="str">
+        <v>生成时间：2026-08-24T06:54:56Z</v>
+      </c>
+      <c r="B35" s="21" t="str">
+        <v/>
+      </c>
+      <c r="C35" s="21" t="str">
+        <v/>
+      </c>
+      <c r="D35" s="21" t="str">
+        <v/>
+      </c>
+      <c r="E35" s="21" t="str">
+        <v/>
+      </c>
+      <c r="F35" s="21" t="str">
+        <v/>
+      </c>
+      <c r="G35" s="21" t="str">
+        <v/>
+      </c>
+      <c r="H35" s="21" t="str">
+        <v/>
+      </c>
+      <c r="I35" s="21" t="str">
+        <v/>
+      </c>
+      <c r="J35" s="21" t="str">
+        <v/>
+      </c>
+      <c r="K35" s="21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="21" t="str">
         <v>说明：一致=与厂商官方价偏差&lt;0.5%；≥50%且未登记例外标「待核验」须人工复核；模型级不一致=任一档位不一致</v>
       </c>
-      <c r="B24" s="21" t="str">
-        <v/>
-      </c>
-      <c r="C24" s="21" t="str">
-        <v/>
-      </c>
-      <c r="D24" s="21" t="str">
-        <v/>
-      </c>
-      <c r="E24" s="21" t="str">
-        <v/>
-      </c>
-      <c r="F24" s="21" t="str">
-        <v/>
-      </c>
-      <c r="G24" s="21" t="str">
-        <v/>
-      </c>
-      <c r="H24" s="21" t="str">
-        <v/>
-      </c>
-      <c r="I24" s="21" t="str">
-        <v/>
-      </c>
-      <c r="J24" s="21" t="str">
-        <v/>
-      </c>
-      <c r="K24" s="21" t="str">
+      <c r="B36" s="21" t="str">
+        <v/>
+      </c>
+      <c r="C36" s="21" t="str">
+        <v/>
+      </c>
+      <c r="D36" s="21" t="str">
+        <v/>
+      </c>
+      <c r="E36" s="21" t="str">
+        <v/>
+      </c>
+      <c r="F36" s="21" t="str">
+        <v/>
+      </c>
+      <c r="G36" s="21" t="str">
+        <v/>
+      </c>
+      <c r="H36" s="21" t="str">
+        <v/>
+      </c>
+      <c r="I36" s="21" t="str">
+        <v/>
+      </c>
+      <c r="J36" s="21" t="str">
+        <v/>
+      </c>
+      <c r="K36" s="21" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K36"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5325,7 +5745,7 @@
         <v>文生图 · 4K</v>
       </c>
       <c r="E10" s="9" t="str">
-        <v>¥0.26/张</v>
+        <v>¥0.1/张</v>
       </c>
       <c r="F10" s="9" t="str">
         <v>¥0.26/张</v>
@@ -5334,7 +5754,7 @@
         <v>$0.0154</v>
       </c>
       <c r="H10" s="9" t="str">
-        <v>✅ 一致</v>
+        <v>⚠+160%</v>
       </c>
       <c r="I10" s="9" t="str">
         <v>⚠+159.7%</v>
@@ -5412,7 +5832,7 @@
         <v>单图生图 · 4K</v>
       </c>
       <c r="E13" s="9" t="str">
-        <v>¥0.26/张</v>
+        <v>¥0.1/张</v>
       </c>
       <c r="F13" s="9" t="str">
         <v>¥0.4/张</v>
@@ -5421,7 +5841,7 @@
         <v>$0.0154</v>
       </c>
       <c r="H13" s="9" t="str">
-        <v>⚠+53.8%</v>
+        <v>⚠+300%</v>
       </c>
       <c r="I13" s="9" t="str">
         <v>⚠+299.6%</v>
@@ -5499,7 +5919,7 @@
         <v>多图参考生图 · 4K</v>
       </c>
       <c r="E16" s="9" t="str">
-        <v>¥0.26/张</v>
+        <v>¥0.1/张</v>
       </c>
       <c r="F16" s="9" t="str">
         <v>¥0.56/张</v>
@@ -5508,7 +5928,7 @@
         <v>$0.0154</v>
       </c>
       <c r="H16" s="9" t="str">
-        <v>⚠+115.4%</v>
+        <v>⚠+460%</v>
       </c>
       <c r="I16" s="9" t="str">
         <v>⚠+459.4%</v>
@@ -5673,7 +6093,7 @@
         <v>4K</v>
       </c>
       <c r="E22" s="9" t="str">
-        <v>¥0.4/张</v>
+        <v>¥0.2/张</v>
       </c>
       <c r="F22" s="9" t="str">
         <v>¥0.4/张</v>
@@ -5682,7 +6102,7 @@
         <v>$0.0616</v>
       </c>
       <c r="H22" s="9" t="str">
-        <v>✅ 一致</v>
+        <v>⚠+100%</v>
       </c>
       <c r="I22" s="9" t="str">
         <v>一致</v>
@@ -5789,7 +6209,7 @@
         <v>4K</v>
       </c>
       <c r="E26" s="9" t="str">
-        <v>¥0.4/张</v>
+        <v>¥0.2/张</v>
       </c>
       <c r="F26" s="9" t="str">
         <v>¥0.4/张</v>
@@ -5798,7 +6218,7 @@
         <v>$0.0616</v>
       </c>
       <c r="H26" s="9" t="str">
-        <v>✅ 一致</v>
+        <v>⚠+100%</v>
       </c>
       <c r="I26" s="9" t="str">
         <v>一致</v>
@@ -7601,7 +8021,7 @@
         <v>文生图 · 4K</v>
       </c>
       <c r="E7" s="7" t="str">
-        <v>¥0.26/张</v>
+        <v>¥0.1/张</v>
       </c>
       <c r="F7" s="7" t="str">
         <v>$0.037/张</v>
@@ -7610,7 +8030,7 @@
         <v>$0.0154</v>
       </c>
       <c r="H7" s="7" t="str">
-        <v>⚠-7.5%</v>
+        <v>⚠+140.5%</v>
       </c>
       <c r="I7" s="7" t="str">
         <v>⚠+140.3%</v>
@@ -7688,7 +8108,7 @@
         <v>单图生图 · 4K</v>
       </c>
       <c r="E10" s="7" t="str">
-        <v>¥0.26/张</v>
+        <v>¥0.1/张</v>
       </c>
       <c r="F10" s="7" t="str">
         <v>$0.056/张</v>
@@ -7697,7 +8117,7 @@
         <v>$0.0154</v>
       </c>
       <c r="H10" s="7" t="str">
-        <v>⚠+40%</v>
+        <v>⚠+264%</v>
       </c>
       <c r="I10" s="7" t="str">
         <v>⚠+263.6%</v>
@@ -7775,7 +8195,7 @@
         <v>多图参考生图 · 4K</v>
       </c>
       <c r="E13" s="7" t="str">
-        <v>¥0.26/张</v>
+        <v>¥0.1/张</v>
       </c>
       <c r="F13" s="7" t="str">
         <v>$0.079/张</v>
@@ -7784,7 +8204,7 @@
         <v>$0.0154</v>
       </c>
       <c r="H13" s="7" t="str">
-        <v>⚠+97.5%</v>
+        <v>⚠+413.5%</v>
       </c>
       <c r="I13" s="7" t="str">
         <v>⚠+413%</v>
@@ -7949,7 +8369,7 @@
         <v>4K</v>
       </c>
       <c r="E19" s="7" t="str">
-        <v>¥0.4/张</v>
+        <v>¥0.2/张</v>
       </c>
       <c r="F19" s="7" t="str">
         <v>$0.056/张</v>
@@ -7958,7 +8378,7 @@
         <v>$0.0616</v>
       </c>
       <c r="H19" s="7" t="str">
-        <v>⚠-9%</v>
+        <v>⚠+82%</v>
       </c>
       <c r="I19" s="7" t="str">
         <v>⚠-9.1%</v>
@@ -8065,7 +8485,7 @@
         <v>4K</v>
       </c>
       <c r="E23" s="7" t="str">
-        <v>¥0.4/张</v>
+        <v>¥0.2/张</v>
       </c>
       <c r="F23" s="7" t="str">
         <v>$0.056/张</v>
@@ -8074,7 +8494,7 @@
         <v>$0.0616</v>
       </c>
       <c r="H23" s="7" t="str">
-        <v>⚠-9%</v>
+        <v>⚠+82%</v>
       </c>
       <c r="I23" s="7" t="str">
         <v>⚠-9.1%</v>

</xml_diff>